<commit_message>
feat: complete ADB CMS integration, 105 genuine collaboration partners, 10-partner outreach pipeline (3,144 drafts), and verified email provider
</commit_message>
<xml_diff>
--- a/backend/storage/Andhra Pradesh/Spatial/2026_AND_1263790_12/BOQ_Financial_Schedule_2026_AND_1263790_12.xlsx
+++ b/backend/storage/Andhra Pradesh/Spatial/2026_AND_1263790_12/BOQ_Financial_Schedule_2026_AND_1263790_12.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="BOQ &amp; Financial Bid" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Item Rate BoQ" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Milestone Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Bidder Declaration" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="5">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0&quot;%&quot;"/>
+  </numFmts>
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,28 +32,58 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001E1B4B"/>
+      <color rgb="000F172A"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="000F172A"/>
+      <color rgb="00334155"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="000F172A"/>
+      <color rgb="001E293B"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="000F172A"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E1B4B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E1B4B"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -58,18 +92,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E1B4B"/>
-        <bgColor rgb="001E1B4B"/>
+        <fgColor rgb="000F172A"/>
+        <bgColor rgb="000F172A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
-        <bgColor rgb="00F1F5F9"/>
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF2FF"/>
+        <bgColor rgb="00EEF2FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0E7FF"/>
+        <bgColor rgb="00E0E7FF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -91,11 +137,25 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="double">
+        <color rgb="001E1B4B"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -106,24 +166,67 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -491,28 +594,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="65" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="68" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BILL OF QUANTITIES (BOQ) — FINANCIAL BID SCHEDULE</t>
+          <t>OFFICIAL GOVERNMENT BILL OF QUANTITIES (BOQ) — FINANCIAL SCHEDULE</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tender Ref: 2026_AND_1263790_12 | Department: PUBLIC WORKS &amp; HIGHWAYS DEPARTMENT</t>
+          <t>Tender Ref: 2026_AND_1263790_12 | Authority: PUBLIC WORKS &amp; HIGHWAYS DEPARTMENT</t>
         </is>
       </c>
     </row>
@@ -523,190 +628,633 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Validate Price Bid: Rates entered by bidder must include all overheads, equipment deployment, field survey, processing &amp; software.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Item No.</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Item Description</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Estimated Rate (INR)</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Total Amount (INR)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Basic Estimated Rate (INR)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Basic Total Amount (INR)</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>GST Rate (%)</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Total Amount with GST (INR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>1.01</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Survey &amp; Primary Data Collection / Field Geo-tagging</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="n">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Mobile LiDAR Scanning (MLS) &amp; 360-degree High-Definition Panoramic Video Road Survey</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Lane-Km</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>6800</v>
+      </c>
+      <c r="F7" s="9">
+        <f>C7*E7</f>
+        <v/>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="H7" s="9">
+        <f>F7*(1+G7/100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>1.02</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Automated Pavement Distress &amp; Roughness Index (IRI) Evaluation using Computer Vision</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Lane-Km</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F8" s="14">
+        <f>C8*E8</f>
+        <v/>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="H8" s="14">
+        <f>F8*(1+G8/100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>1.03</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>3D Road Asset Feature Extraction (Signboards, Streetlights, Bridges, Culverts, Footpaths)</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Lane-Km</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>5200</v>
+      </c>
+      <c r="F9" s="9">
+        <f>C9*E9</f>
+        <v/>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="H9" s="9">
+        <f>F9*(1+G9/100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Road Network Spatial Geodatabase Creation adhering to IRC:SP:19 and IRC:SP:84 guidelines</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>Job</t>
         </is>
       </c>
-      <c r="E6" s="8" t="n">
-        <v>450000</v>
-      </c>
-      <c r="F6" s="8" t="n">
-        <v>450000</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>1.02</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>High-Resolution Spatial Data Processing &amp; Ortho-mosaic Mapping</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="n">
+      <c r="E10" s="14" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="F10" s="14">
+        <f>C10*E10</f>
+        <v/>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="H10" s="14">
+        <f>F10*(1+G10/100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>1.05</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Enterprise Pavement Management System (PMS) Web Portal &amp; GIS Decision Support System</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="F11" s="9">
+        <f>C11*E11</f>
+        <v/>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="H11" s="9">
+        <f>F11*(1+G11/100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Periodic Maintenance Schedule Formulation and Priority Defect Matrix Report</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>Job</t>
         </is>
       </c>
-      <c r="E7" s="8" t="n">
-        <v>620000</v>
-      </c>
-      <c r="F7" s="8" t="n">
-        <v>620000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>1.03</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Enterprise Web GIS Platform Development &amp; Cloud Infrastructure</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>System</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F8" s="8" t="n">
-        <v>850000</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>1.04</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Integration with Existing State e-Governance Portals and Databases</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Lump-sum</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="n">
-        <v>380000</v>
-      </c>
-      <c r="F9" s="8" t="n">
-        <v>380000</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>1.05</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Comprehensive Operations, Technical Support &amp; Maintenance (1 Year)</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="E12" s="14" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="F12" s="14">
+        <f>C12*E12</f>
+        <v/>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="H12" s="14">
+        <f>F12*(1+G12/100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Cloud Server Hosting, Annual Data Updates and Multi-Year Facility Management Support</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Months</t>
         </is>
       </c>
-      <c r="E10" s="8" t="n">
-        <v>45000</v>
-      </c>
-      <c r="F10" s="8" t="n">
-        <v>540000</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>TOTAL ESTIMATED CONTRACT VALUE (INR)</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="11">
-        <f>SUM(F6:F10)</f>
+      <c r="E13" s="9" t="n">
+        <v>110000</v>
+      </c>
+      <c r="F13" s="9">
+        <f>C13*E13</f>
+        <v/>
+      </c>
+      <c r="G13" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="H13" s="9">
+        <f>F13*(1+G13/100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>SUB-TOTAL BASIC CONTRACT VALUE (INR)</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="n"/>
+      <c r="C14" s="17" t="n"/>
+      <c r="D14" s="17" t="n"/>
+      <c r="E14" s="17" t="n"/>
+      <c r="F14" s="18">
+        <f>SUM(F7:F13)</f>
+        <v/>
+      </c>
+      <c r="G14" s="17" t="n"/>
+      <c r="H14" s="17" t="n"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>APPLICABLE GOODS &amp; SERVICES TAX (GST @ 18%) (INR)</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="n"/>
+      <c r="C15" s="17" t="n"/>
+      <c r="D15" s="17" t="n"/>
+      <c r="E15" s="17" t="n"/>
+      <c r="F15" s="18">
+        <f>F14*0.18</f>
+        <v/>
+      </c>
+      <c r="G15" s="17" t="n"/>
+      <c r="H15" s="17" t="n"/>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>TOTAL ESTIMATED TENDER VALUE INCLUSIVE OF ALL TAXES (INR)</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="n"/>
+      <c r="C16" s="20" t="n"/>
+      <c r="D16" s="20" t="n"/>
+      <c r="E16" s="20" t="n"/>
+      <c r="F16" s="21">
+        <f>F14+F15</f>
+        <v/>
+      </c>
+      <c r="G16" s="20" t="n"/>
+      <c r="H16" s="21">
+        <f>F16</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A11:E11"/>
+  <mergeCells count="7">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A14:E14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>PROJECT DELIVERABLE MILESTONES &amp; DISBURSEMENT PERCENTAGES</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="23" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>Deliverable Scope</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="inlineStr">
+        <is>
+          <t>Timeline</t>
+        </is>
+      </c>
+      <c r="D3" s="23" t="inlineStr">
+        <is>
+          <t>Payment Share (%)</t>
+        </is>
+      </c>
+      <c r="E3" s="23" t="inlineStr">
+        <is>
+          <t>Cumulative (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>M-1</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>Inception Report, Project Quality Plan &amp; Statutory Clearances</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>T0 + 30 Days</t>
+        </is>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" s="26" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>M-2</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>DGPS Ground Control Network, Flight Survey &amp; Raw Sensor Verification</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>T0 + 90 Days</t>
+        </is>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>20</v>
+      </c>
+      <c r="E5" s="26" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>M-3</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>Ortho-mosaic Processing, Feature Extraction &amp; 50% Field Verification</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>T0 + 180 Days</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>25</v>
+      </c>
+      <c r="E6" s="26" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>M-4</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>100% Survey Completion, UPIN Geo-tagging &amp; Database Validation</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>T0 + 270 Days</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>25</v>
+      </c>
+      <c r="E7" s="26" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>M-5</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="inlineStr">
+        <is>
+          <t>Web GIS Portal Deployment, User Acceptance Testing (UAT) &amp; Training</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>T0 + 330 Days</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="26" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>M-6</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="inlineStr">
+        <is>
+          <t>Final Handover Sign-off &amp; Commencement of AMC / Operations</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>T0 + 365 Days</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" s="26" t="n">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>STATUTORY UNDERTAKING BY COMMERCIAL BIDDER</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1. We confirm that the rates quoted above in the Item Rate BoQ are complete and inclusive of all taxes,</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   duties, levies, transportation, insurance, survey sensor equipment, software licenses, and field manpower.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2. The financial proposal shall remain valid for 180 calendar days from the date of technical bid opening.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>3. We understand that mathematical formulas in the official Excel BOQ are automated and verify all calculations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4. In case of any mathematical discrepancy between unit rates and total amount, unit rates shall prevail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Name of Authorized Signatory: ________________________________________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Designation: _______________________________________________________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Company Seal &amp; Digital Signature: ___________________________________________</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>